<commit_message>
feat: add invoice dual-scope workbench
</commit_message>
<xml_diff>
--- a/tests/fixtures/synthetic_base.xlsx
+++ b/tests/fixtures/synthetic_base.xlsx
@@ -697,7 +697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A4:AE9"/>
+  <dimension ref="A4:U9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="4">
@@ -798,62 +798,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2601</t>
+          <t>SHIP QTY</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>2602</t>
-        </is>
-      </c>
-      <c r="V4" t="inlineStr">
-        <is>
-          <t>2603</t>
-        </is>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>2604</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>2605</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>2606</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>2607</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>2608</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr">
-        <is>
-          <t>2609</t>
-        </is>
-      </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t>2610</t>
-        </is>
-      </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>2611</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr">
-        <is>
-          <t>2612</t>
+          <t>BALANCE QTY</t>
         </is>
       </c>
     </row>
@@ -1060,6 +1010,9 @@
       <c r="T7" t="n">
         <v>360</v>
       </c>
+      <c r="U7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1093,7 +1046,7 @@
         </is>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="H8" t="n">
         <v>28</v>
@@ -1123,8 +1076,11 @@
       <c r="S8" t="n">
         <v>24</v>
       </c>
-      <c r="V8" t="n">
+      <c r="T8" t="n">
         <v>100</v>
+      </c>
+      <c r="U8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1171,6 +1127,12 @@
       </c>
       <c r="S9" t="n">
         <v>24</v>
+      </c>
+      <c r="T9" t="n">
+        <v>50</v>
+      </c>
+      <c r="U9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>